<commit_message>
Feat :Delivery date,Pricing engine,Order splitting into jobs,Order confirmation,File
</commit_message>
<xml_diff>
--- a/documentation/capstone/planning/PrintGrid-Ke-hoach-1-Trang.xlsx
+++ b/documentation/capstone/planning/PrintGrid-Ke-hoach-1-Trang.xlsx
@@ -3,6 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500"/>
+  </bookViews>
   <sheets>
     <sheet sheetId="1" name="PHÂN CÔNG — 1 TRANG" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Tải 4 người" state="visible" r:id="rId5"/>
@@ -12,9 +15,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="357">
-  <si>
-    <t>MỘT TRANG DUY NHẤT — xếp theo Tuần 1→8. CỔNG G-A (cuối T2): một đơn chạy hết chuỗi bằng cầu đánh dấu-đã-trả, không nhờ dữ liệu mẫu. CỔNG G-B (T8): bảng 16 chỉ số đạt + SEPay sandbox + 3 màn diễn tập. Quy tắc chọn việc: một thư mục FE — một tuần — một người; bắt tay qua hợp đồng API/event, không sửa file của nhau (xem bảng cuối sheet). SRS: documentation/project/requirements/ 09·12·13.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="652" uniqueCount="397">
+  <si>
+    <t>MỘT TRANG DUY NHẤT — xếp theo Tuần 1→8. CỔNG G-A (cuối T2): một đơn chạy hết chuỗi bằng cầu đánh dấu-đã-trả, không nhờ dữ liệu mẫu. CỔNG G-B (T8): bảng 16 chỉ số đạt + SEPay sandbox + 3 màn diễn tập. Quy tắc chọn việc: một thư mục FE — một tuần — một người; bắt tay qua hợp đồng API/event, không sửa file của nhau (xem bảng cuối sheet). SRS: documentation/project/requirements/ 09·12·13. REVIEW 1 (30/09): 🆕R1 = việc mới thêm; 🔧R1 = việc cũ đã sửa theo kết luận; ❌R1 = ứng viên cắt. BCD nâng 8 entity (gộp chờ B25) — sơ đồ vẽ lại sau khi GVHD duyệt.</t>
   </si>
   <si>
     <t>STT</t>
@@ -53,7 +56,7 @@
     <t>Nền</t>
   </si>
   <si>
-    <t>Thống nhất hợp đồng API và nền móng repo chung</t>
+    <t>Họp khóa hợp đồng + nền repo</t>
   </si>
   <si>
     <t>Cả nhóm</t>
@@ -77,7 +80,7 @@
     <t>AC01: openapi.yaml có Order/Quote/Job/Slot/event; AC02: docker compose up — 2 máy khác nhau gọi lẫn nhau thành công</t>
   </si>
   <si>
-    <t>Gỡ toàn bộ dữ liệu mẫu khỏi hệ thống</t>
+    <t>Dọn dữ liệu mẫu</t>
   </si>
   <si>
     <t>đăng nhập, trang đơn</t>
@@ -95,7 +98,7 @@
     <t>S8</t>
   </si>
   <si>
-    <t>Tính đúng kích thước, thể tích, lỗi của mô hình in 3D</t>
+    <t>Phân tích hình học model</t>
   </si>
   <si>
     <t>Hệ thống</t>
@@ -113,7 +116,7 @@
     <t>AC01: cube 10 mm → bbox 10×10×10; AC02: file rỗng/rác → báo lỗi chỉ rõ nguyên nhân; AC03: &lt;10 giây</t>
   </si>
   <si>
-    <t>Ước lượng thời gian in và vật liệu tiêu hao</t>
+    <t>Ước lượng thời gian + vật liệu</t>
   </si>
   <si>
     <t>đơn-config (trạng thái xử lý)</t>
@@ -131,7 +134,7 @@
     <t>S1</t>
   </si>
   <si>
-    <t>Bảng người dùng và phân quyền thật thay hardcode</t>
+    <t>Bảng người dùng + vai thật</t>
   </si>
   <si>
     <t>Admin</t>
@@ -149,7 +152,7 @@
     <t>AC01: tạo user Lab trong DB → login vào đúng trang Lab; AC02: DemoRoles.cs không còn tham chiếu</t>
   </si>
   <si>
-    <t>Xác minh email khi khách đăng ký</t>
+    <t>Xác thực email</t>
   </si>
   <si>
     <t>Khách hàng</t>
@@ -170,7 +173,7 @@
     <t>S3</t>
   </si>
   <si>
-    <t>Kiểm tra và báo sớm mô hình không in được</t>
+    <t>Cảnh báo model không in được</t>
   </si>
   <si>
     <t>thư viện model · đơn-config</t>
@@ -185,7 +188,7 @@
     <t>AC01: model 400 mm → không bấm được "Lấy báo giá"; AC02: thông báo nêu khổ lớn nhất mạng</t>
   </si>
   <si>
-    <t>Báo giá với ngày giao tính theo lịch máy thực tế</t>
+    <t>Ngày giao từ năng lực thật</t>
   </si>
   <si>
     <t>đơn-config (chip kết quả)</t>
@@ -197,10 +200,13 @@
     <t>FR-SCHED-005 · BR-QUOTE-002, SCHED-001 · PERF-001</t>
   </si>
   <si>
-    <t>AC01: dựng 2 lab trống vs đầy ⇒ 2 ngày khác nhau; AC02: ngày in lại ≠ hằng số +3; AC03: ≤60 giây</t>
-  </si>
-  <si>
-    <t>Định giá thống nhất, khóa phiên bản bảng giá vào báo giá</t>
+    <t>Xong</t>
+  </si>
+  <si>
+    <t>AC01: dựng 2 lab trống vs đầy ⇒ 2 ngày khác nhau; AC02: ngày in lại ≠ hằng số +3; AC03: ≤60 giây ✔ code 02/10, smoke pass</t>
+  </si>
+  <si>
+    <t>Máy định giá đóng băng kỳ giá</t>
   </si>
   <si>
     <t>admin/cấu hình giá (T4 hiển thị)</t>
@@ -212,10 +218,10 @@
     <t>FR-SCHED-010 · BR-QUOTE-001..004 · MAINT-005</t>
   </si>
   <si>
-    <t>AC01: tổng breakdown = giá; AC02: đổi giá xong báo giá cũ tính lại giữ nguyên; AC03: cùng cấu hình ⇒ cùng giá</t>
-  </si>
-  <si>
-    <t>Chia đơn thành công việc in, xếp lịch không chồng chéo</t>
+    <t>AC01: tổng breakdown = giá; AC02: đổi giá xong báo giá cũ tính lại giữ nguyên; AC03: cùng cấu hình ⇒ cùng giá ✔ code 02/10, smoke pass</t>
+  </si>
+  <si>
+    <t>Tách đơn thành job, không trùng lịch</t>
   </si>
   <si>
     <t>— (engine) · lab queue thấy kết quả</t>
@@ -227,13 +233,13 @@
     <t>FR-SCHED-006 · BR-SCHED-001..004 · REL-004</t>
   </si>
   <si>
-    <t>AC01: 10 worker đặt song song ⇒ 0 slot chồng; AC02: job có due ≤ ngày giao trừ hub+ship; AC03: bỏ hằng số demo 120³</t>
+    <t>AC01: 10 worker đặt song song ⇒ 0 slot chồng; AC02: job có due ≤ ngày giao trừ hub+ship; AC03: bỏ hằng số demo 120³ ✔ code 02/10, smoke pass</t>
   </si>
   <si>
     <t>S4</t>
   </si>
   <si>
-    <t>Xác nhận đơn hàng kèm điều khoản sử dụng</t>
+    <t>Xác nhận đơn + điều khoản</t>
   </si>
   <si>
     <t>đơn-config (bước cuối)</t>
@@ -245,10 +251,10 @@
     <t>FR-CUST-007 · BR-QUOTE-003, PAY-001</t>
   </si>
   <si>
-    <t>AC01: không tick ⇒ nút disable; AC02: báo giá hết hạn ⇒ không tạo đơn</t>
-  </si>
-  <si>
-    <t>Chế độ tạm: vận hành xác nhận đã thu tiền để đơn chạy tiếp</t>
+    <t>AC01: không tick ⇒ nút disable; AC02: báo giá hết hạn ⇒ không tạo đơn ✔ code 02/10, smoke pass</t>
+  </si>
+  <si>
+    <t>Cầu tạm đánh dấu đã trả 🔧R1 (nay = phần CỌC)</t>
   </si>
   <si>
     <t>Quản trị mạng</t>
@@ -269,7 +275,7 @@
     <t>S6</t>
   </si>
   <si>
-    <t>Xưởng nhận hoặc từ chối việc trong hạn 2 giờ</t>
+    <t>Nhận offer + accept/từ chối hạn 2 giờ 🔧R1</t>
   </si>
   <si>
     <t>Quản lý xưởng</t>
@@ -278,19 +284,34 @@
     <t>lab/hàng đợi job</t>
   </si>
   <si>
-    <t>Từ chối chọn lý do; đếm giờ; quá hạn tự nhả về engine</t>
-  </si>
-  <si>
-    <t>FR-LAB-004 · BR-ASSIGN-005/006</t>
+    <t>Fan-out top-k offer (BR-ASSIGN-010); từ chối có lý do; đếm giờ; accept phải kèm xác nhận hash file</t>
+  </si>
+  <si>
+    <t>FR-LAB-004 · BR-ASSIGN-005/006/010, IP-003</t>
   </si>
   <si>
     <t>AC01: từ chối ⇒ job về pending trong ≤5 phút; AC02: đồng hồ hiện đúng hạn còn lại</t>
   </si>
   <si>
+    <t>🆕R1 Băm file + email bằng chứng</t>
+  </si>
+  <si>
+    <t>thư viện model (sau tải lên)</t>
+  </si>
+  <si>
+    <t>SHA-256 lúc nhận, lưu metadata; email xác nhận (thời gian, tên, dung lượng, hash); accept job tích xác nhận hash khớp</t>
+  </si>
+  <si>
+    <t>FR-CUST-002b · BR-IP-001..003 · LEGAL-003</t>
+  </si>
+  <si>
+    <t>AC01: upload ⇒ hash + email ≤1 phút; AC02: 2 file lệch 1 byte ⇒ hash khác, hệ thống báo; AC03: tra tranh chấp ra đủ file/hash/thời gian/người gửi-người nhận ✔ code 02/10, smoke pass</t>
+  </si>
+  <si>
     <t>S7</t>
   </si>
   <si>
-    <t>Hub tiếp nhận lô hàng, đối chiếu đủ thiếu</t>
+    <t>Hub nhận lô đối chiếu</t>
   </si>
   <si>
     <t>QC hub</t>
@@ -308,7 +329,7 @@
     <t>AC01: lô 3 job báo 2 ⇒ 1 dòng MISSING + thông báo xưởng; AC02: nhận xong đẩy vào hàng đợi kiểm</t>
   </si>
   <si>
-    <t>Tập hợp đơn, đóng gói, gửi hàng, xác nhận giao</t>
+    <t>Gộp đơn, pack, ship, giao</t>
   </si>
   <si>
     <t>Thủ kho hub</t>
@@ -329,7 +350,7 @@
     <t>S5</t>
   </si>
   <si>
-    <t>Khách theo dõi đơn theo thời gian thực</t>
+    <t>Theo dõi đơn realtime</t>
   </si>
   <si>
     <t>đơn hàng (timeline)</t>
@@ -344,7 +365,7 @@
     <t>AC01: thợ bấm "đang in" ⇒ tab khách đổi ≤15 giây; AC02: soi payload 0 chữ lab</t>
   </si>
   <si>
-    <t>Bổ sung đủ lựa chọn cấu hình in</t>
+    <t>Đủ thông số in</t>
   </si>
   <si>
     <t>đơn-config (cấu hình)</t>
@@ -359,7 +380,7 @@
     <t>AC01: chọn resin không tồn kho ⇒ disable có lý do; AC02: các field mới vào báo giá</t>
   </si>
   <si>
-    <t>Màn hình báo giá hiển thị số thật từ hệ thống</t>
+    <t>Màn báo giá số thật</t>
   </si>
   <si>
     <t>đơn-config (báo giá)</t>
@@ -371,10 +392,10 @@
     <t>FR-CUST-006 · BR-QUOTE-005/007 · PERF-001</t>
   </si>
   <si>
-    <t>AC01: số màn = số API; AC02: hạn 48h chạy thật; AC03: FE không tự tính giá</t>
-  </si>
-  <si>
-    <t>Bộ kiểm thử tích hợp chạy tự động trên CI</t>
+    <t>AC01: số màn = số API; AC02: hạn 48h chạy thật; AC03: FE không tự tính giá ✔ code 02/10, smoke pass</t>
+  </si>
+  <si>
+    <t>Kiểm thử tích hợp tự động</t>
   </si>
   <si>
     <t>—</t>
@@ -389,27 +410,72 @@
     <t>AC01: dotnet test xanh; AC02: ca song song là regression cho AC01 task tuần 2</t>
   </si>
   <si>
-    <t>Hệ thống tự xếp lại lịch khi có sự cố</t>
+    <t>Tự vá lịch khi biến cố</t>
   </si>
   <si>
     <t>— (engine) · ops/monitor T4</t>
   </si>
   <si>
-    <t>Xử lý từ-chối/in-hỏng/chết-máy ≤30s; không đụng đang in; lịch dự phòng; không kịp ⇒ luồng xin dời</t>
-  </si>
-  <si>
-    <t>FR-SCHED-007 · BR-RESCHED-001/002, SCHED-005..008 · PERF-002</t>
+    <t>Xử lý từ-chối/in-hỏng/chết-máy ≤30s; không đụng đang in; lịch dự phòng; ưu tiên: split lô → gán lại → xin dời ngày (BR-SCHED-010/011)</t>
+  </si>
+  <si>
+    <t>FR-SCHED-007 · BR-RESCHED-001/002, SCHED-005..008/010/011 · PERF-002</t>
   </si>
   <si>
     <t>AC01: fail ở 80% thời lượng ⇒ job khác máy ≤30s; AC02: 0 job IN_PROGRESS bị đổi; AC03: khách không trễ nếu còn slack</t>
   </si>
   <si>
-    <t>In lại khẩn giữ ngày giao gốc, quá 2 lần thì báo người</t>
+    <t>🆕R1 Chia lô khi đe dọa trễ</t>
   </si>
   <si>
     <t>— (engine)</t>
   </si>
   <si>
+    <t>Item số lượng lớn forecast trễ ⇒ tách ≥2 lab cùng làm, giá không đổi; không cứu được ⇒ sinh đề nghị dời ngày</t>
+  </si>
+  <si>
+    <t>FR-SCHED-010 · BR-SCHED-010/011, QUOTE-001</t>
+  </si>
+  <si>
+    <t>AC01: 100 sp quá tải 1 lab ⇒ chia ≥2 lab, ngày ≤ cam kết; AC02: không đủ ⇒ Date-Change Request tự tạo</t>
+  </si>
+  <si>
+    <t>🆕R1 Duyệt ảnh chứng QC xưởng</t>
+  </si>
+  <si>
+    <t>Order Staff</t>
+  </si>
+  <si>
+    <t>staff/chứng-minh</t>
+  </si>
+  <si>
+    <t>Hàng đợi ảnh + báo cáo tự kiểm từ xưởng; đạt ⇒ mở khóa bàn giao; không đạt ⇒ trả kèm lý do</t>
+  </si>
+  <si>
+    <t>FR-ANAL-007 · BR-QC-011/012</t>
+  </si>
+  <si>
+    <t>AC01: chưa duyệt ⇒ API handover 409; AC02: mỗi quyết định audit người/thời gian/lý do</t>
+  </si>
+  <si>
+    <t>🆕R1 Bàn duyệt báo giá nháp ⇒ công bố</t>
+  </si>
+  <si>
+    <t>staff/báo-giá-nháp</t>
+  </si>
+  <si>
+    <t>Engine draft; chỉnh trong băng + lý do; auto-lane dưới ngưỡng cfg; hạn báo giá tính từ lúc duyệt</t>
+  </si>
+  <si>
+    <t>FR-ANAL-006 · BR-QUOTE-008/003 · PERF-001</t>
+  </si>
+  <si>
+    <t>AC01: draft chưa duyệt khách không thấy; AC02: ngoài băng ⇒ chặn; AC03: ⚠B23 chốt ngưỡng auto-lane</t>
+  </si>
+  <si>
+    <t>In lại khẩn lịch gốc, chặn quá 2</t>
+  </si>
+  <si>
     <t>URGENT deadline gốc; phí theo bên lỗi; lần 3 ⇒ hàng đợi vận hành</t>
   </si>
   <si>
@@ -419,7 +485,7 @@
     <t>AC01: job in lại có deadline = gốc; AC02: lần 3 không tự chạy, có dòng chờ ops</t>
   </si>
   <si>
-    <t>Lưu vết từng quyết định chọn xưởng in</t>
+    <t>Nhật ký quyết định gán</t>
   </si>
   <si>
     <t>ops/hạch-thực-gán (T4 màn)</t>
@@ -434,7 +500,7 @@
     <t>AC01: tra job bất kỳ ra ≥1 ứng viên + điểm; AC02: tắt bảng log ⇒ gán thất bại toàn bộ (không im lặng)</t>
   </si>
   <si>
-    <t>Lọc máy in theo đủ mọi điều kiện khả thi</t>
+    <t>Lọc khả thi đủ ràng buộc</t>
   </si>
   <si>
     <t>Thêm tồn kho + uy tín; 30 ca cố-ý-không-khả-thi, test tách scoring</t>
@@ -446,22 +512,22 @@
     <t>AC01: 0 vi phạm trong suite; AC02: stock = 0 ⇒ lab mất tổ hợp màu</t>
   </si>
   <si>
-    <t>Quản lý kho vật liệu theo màu và số lượng</t>
+    <t>Kho vật liệu dạng sổ 🔧R1</t>
   </si>
   <si>
     <t>lab/kho</t>
   </si>
   <si>
-    <t>Giữ khi nhận job, quyết toán khi xong; cảnh báo gần hết</t>
-  </si>
-  <si>
-    <t>FR-LAB-003 · BR-ASSIGN-001</t>
+    <t>Giữ khi nhận job (+1–5% dung sai), quyết toán số thực; mỗi nhập-xuất = một mã giao dịch chạy lũy kế; cảnh báo gần hết</t>
+  </si>
+  <si>
+    <t>FR-LAB-003 · BR-ASSIGN-001, STOCK-001..003</t>
   </si>
   <si>
     <t>AC01: nhận job 50 g ⇒ kho trừ 50; AC02: dưới ngưỡng ⇒ cảnh báo + engine không giao thêm màu đó</t>
   </si>
   <si>
-    <t>Màn hình vận hành in thân thiện với xưởng</t>
+    <t>Vận hành in chuẩn xưởng</t>
   </si>
   <si>
     <t>Thợ in</t>
@@ -479,7 +545,7 @@
     <t>AC01: tablet 768px thao tác đủ; AC02: hoàn thành thiếu thời gian ⇒ không lưu; AC03: sự cố đẩy sang engine (phối hợp task vá lịch)</t>
   </si>
   <si>
-    <t>Kiểm hàng theo checklist chuẩn</t>
+    <t>Kiểm hàng chuẩn</t>
   </si>
   <si>
     <t>hub/kiểm hàng</t>
@@ -494,7 +560,7 @@
     <t>AC01: không ảnh ⇒ không lưu kết luận; AC02: mỗi mục kiểm có đậu/trượt/không áp dụng; AC03: trượt thiếu quy trách ⇒ không chuyển in lại</t>
   </si>
   <si>
-    <t>Hàng không đạt tự sinh lệnh in lại</t>
+    <t>Kiểm trượt ⇒ in lại</t>
   </si>
   <si>
     <t>Trượt do xưởng/hub ⇒ sự cố sang engine; do khách ⇒ xin khách trả phí</t>
@@ -506,7 +572,7 @@
     <t>AC01: FAIL + lỗi xưởng ⇒ job URGENT xuất hiện ở lab; AC02: lỗi khách ⇒ email gửi, 0 job tạo</t>
   </si>
   <si>
-    <t>Khách gửi yêu cầu in lại hoặc khiếu nại</t>
+    <t>Xin in lại/khiếu nại</t>
   </si>
   <si>
     <t>đơn hàng (sau giao)</t>
@@ -521,7 +587,7 @@
     <t>AC01: ngày 31 ⇒ bị chặn kèm lý do; AC02: gửi xong thấy trạng thái "chờ xử lý"</t>
   </si>
   <si>
-    <t>Thư viện mô hình và thông tin tài khoản khách</t>
+    <t>Thư viện + hồ sơ khách</t>
   </si>
   <si>
     <t>khách/thư viện · hồ sơ-địa-chỉ</t>
@@ -536,7 +602,7 @@
     <t>AC01: reorder điền sẵn config lần trước; AC02: xóa địa chỉ đơn đang chạy ⇒ 409</t>
   </si>
   <si>
-    <t>Kiểm định dạng file và hạn mức dung lượng tải lên</t>
+    <t>Chặt định dạng + quota upload</t>
   </si>
   <si>
     <t>khách/tải file</t>
@@ -551,7 +617,7 @@
     <t>AC01: .exe đổi đuôi .stl ⇒ từ chối; AC02: file 51 MB ⇒ 413 rõ lời</t>
   </si>
   <si>
-    <t>Ghi nhật ký thao tác và màn hình tra cứu</t>
+    <t>Nhật ký hệ thống + màn xem</t>
   </si>
   <si>
     <t>admin/nhật-ký</t>
@@ -566,7 +632,7 @@
     <t>AC01: đổi 1 tham số ⇒ 1 dòng log trước/sau; AC02: API sửa log ⇒ 405; AC03: tra &lt;2 giây</t>
   </si>
   <si>
-    <t>Quản lý người dùng và áp phân quyền mọi API</t>
+    <t>Màn người dùng + RBAC mọi API</t>
   </si>
   <si>
     <t>admin/người-dùng</t>
@@ -584,7 +650,7 @@
     <t>S2</t>
   </si>
   <si>
-    <t>Màn cấu hình tham số kinh doanh có phiên bản</t>
+    <t>Cấu hình thương mại phiên bản</t>
   </si>
   <si>
     <t>admin/cấu-hình</t>
@@ -599,7 +665,7 @@
     <t>AC01: đổiPLA 450→500, quote mới đổi ≤1 phút, quote cũ giữ; AC02: preview trước khi lưu</t>
   </si>
   <si>
-    <t>Đưa danh mục vật liệu, màu, công nghệ vào cơ sở dữ liệu</t>
+    <t>Danh mục dùng chung</t>
   </si>
   <si>
     <t>admin/danh-mục</t>
@@ -614,7 +680,7 @@
     <t>AC01: xóa vật liệu đang ở báo giá ⇒ bị chặn; AC02: thêm PETG-Grey ⇒ hiện ở đơn-config không sửa code</t>
   </si>
   <si>
-    <t>Quản lý checklist kiểm hàng và danh mục lỗi</t>
+    <t>Bộ kiểm + danh mục lỗi</t>
   </si>
   <si>
     <t>admin/bộ-kiểm-hàng</t>
@@ -629,7 +695,7 @@
     <t>AC01: ca kiểm đang chạy giữ phiên bản cũ; AC02: thử xóa mã lỗi đã dùng ⇒ 409</t>
   </si>
   <si>
-    <t>Xưởng tự đăng ký, quản trị viên xét duyệt</t>
+    <t>Xưởng tự đăng ký + duyệt</t>
   </si>
   <si>
     <t>lab/đăng-ký · admin/duyệt</t>
@@ -644,7 +710,7 @@
     <t>AC01: lab chưa duyệt không nhận job; AC02: thiếu máy ⇒ không nộp được</t>
   </si>
   <si>
-    <t>Màn hình khai báo và bảo trì máy in</t>
+    <t>Màn khai máy</t>
   </si>
   <si>
     <t>lab/máy</t>
@@ -659,7 +725,7 @@
     <t>AC01: offline ⇒ filter loại trong ≤1 phút; AC02: xóa máy còn job ⇒ 409</t>
   </si>
   <si>
-    <t>Lịch hoạt động máy và điểm hiệu năng của xưởng</t>
+    <t>Lịch máy + điểm xưởng ❌R1-cắt-candidate</t>
   </si>
   <si>
     <t>lab/dòng-thời-gian · điểm</t>
@@ -674,10 +740,37 @@
     <t>AC01: hoàn tất job ⇒ slot biến mất khỏi tương lai; AC02: điểm hiện đúng 4 chỉ số + mốc so sánh ẩn danh</t>
   </si>
   <si>
+    <t>🆕R1 Gộp nhiều đơn cùng khách một kiện</t>
+  </si>
+  <si>
+    <t>Cùng khách + cùng địa chỉ, ready trong ≤24h ⇒ một vận đơn một kiện; khiếu nại/hoàn vẫn theo đơn gốc</t>
+  </si>
+  <si>
+    <t>FR-HUB-006 · BR-LOG-001/002</t>
+  </si>
+  <si>
+    <t>AC01: 2 đơn cùng khách ⇒ pack gợi ý kiện gộp; AC02: hoàn tiền đúng phạm vi đơn gốc</t>
+  </si>
+  <si>
+    <t>🆕R1 Lô chuyến xưởng → hub</t>
+  </si>
+  <si>
+    <t>lab/lô-chuyến</t>
+  </si>
+  <si>
+    <t>Job đã duyệt chứng tích theo lịch xe; seal ⇒ preview khối lượng + phí zone</t>
+  </si>
+  <si>
+    <t>FR-LAB-008 · BR-LOG-005/003</t>
+  </si>
+  <si>
+    <t>AC01: 3 job xong cùng xưởng ⇒ 1 lô 1 vận đơn; AC02: job gấp ⇒ release ngoại lệ có lý do</t>
+  </si>
+  <si>
     <t>S9</t>
   </si>
   <si>
-    <t>Bảng điều hành mạng lưới và công cụ can thiệp</t>
+    <t>Bảng vận hành + can thiệp</t>
   </si>
   <si>
     <t>ops/monitor · gạch-thực-gán · ghi-lại</t>
@@ -692,7 +785,7 @@
     <t>AC01: job slack&lt;4h đỏ trong ≤15 phút; AC02: gán vào máy không đủ khổ ⇒ 400; AC03: mọi can thiệp có audit</t>
   </si>
   <si>
-    <t>Đọc trọng số chấm điểm từ cấu hình, bỏ mã cứng</t>
+    <t>Bỏ hardcode trọng số</t>
   </si>
   <si>
     <t>Trọng số đọc kỳ cấu hình; đơn vị hồi quy</t>
@@ -704,7 +797,7 @@
     <t>AC01: đổi trọng số tải ⇒ gán kế tiếp đổi theo; AC02: tổng ≠ 1.0 ⇒ chặn lưu</t>
   </si>
   <si>
-    <t>Xin khách đồng ý khi buộc phải dời ngày giao</t>
+    <t>Luồng xin dời ngày</t>
   </si>
   <si>
     <t>khách/link thông-báo</t>
@@ -722,7 +815,7 @@
     <t>S10</t>
   </si>
   <si>
-    <t>Xây hệ thống mô phỏng toàn mạng xưởng in</t>
+    <t>Trạm mô phỏng toàn mạng</t>
   </si>
   <si>
     <t>Nhóm Engine</t>
@@ -740,7 +833,7 @@
     <t>AC01: 2 lần cùng seed khác thời gian ⇒ log giống hệt; AC02: 1000 đơn/tháng chạy hết</t>
   </si>
   <si>
-    <t>Mô phỏng 4 loại sự cố sản xuất thực tế</t>
+    <t>Bơm 4 loại lỗi</t>
   </si>
   <si>
     <t>Từ-chối; hỏng theo % (đỉnh 60–90%); chết máy + thời gian sửa; kiểm trượt</t>
@@ -752,7 +845,7 @@
     <t>AC01: từng loại bật/tắt độc lập bằng config; AC02: hỏng ⇒ vá lịch của T3 bắt buộc chạy</t>
   </si>
   <si>
-    <t>Xem trước mô hình 3D trên trình duyệt (tùy chọn)</t>
+    <t>Xem trước 3D (nên làm)</t>
   </si>
   <si>
     <t>khách/xem-trước-3D</t>
@@ -767,7 +860,7 @@
     <t>AC01: thông số bằng đúng bảng phân tích; AC02: 60 fps trên máy bàn; SẼ CẮT nếu trễ</t>
   </si>
   <si>
-    <t>Đo 4 chiến lược xếp lịch và thử tải quy mô lớn</t>
+    <t>Đo 4 chiến lược + stress</t>
   </si>
   <si>
     <t>4 chiến lược cùng dữ liệu vào; chỉ số trễ đúng hẹn Gini; stress 50 lab/300 máy</t>
@@ -779,7 +872,22 @@
     <t>AC01: bảng 4 cột số; AC02: stress không vỡ cam kết 30s; AC03: mọi số trace về seed</t>
   </si>
   <si>
-    <t>Tự hiệu chỉnh sai lệch ước lượng từ dữ liệu in thật</t>
+    <t>🆕R1 Ghi nhận nhu cầu thiết kế</t>
+  </si>
+  <si>
+    <t>khách/gửi-yêu-cầu</t>
+  </si>
+  <si>
+    <t>Form ý tưởng + ảnh ⇒ queue ops; báo giá nhiều giai đoạn (dùng máy FR-CUST-012); file bàn giao thuộc khách, cấm tái sử dụng</t>
+  </si>
+  <si>
+    <t>FR-CUST-013 · BR-IP-004</t>
+  </si>
+  <si>
+    <t>AC01: yêu cầu vào queue có trạng thái; AC02: sản phẩm gắn draft đơn (thiết kế = runbook)</t>
+  </si>
+  <si>
+    <t>Tự hiệu chỉnh ước lượng</t>
   </si>
   <si>
     <t>ops/monitor (MAPE)</t>
@@ -794,7 +902,7 @@
     <t>AC01: 12 mẫu ⇒ kỳ mới + MAPE giảm; AC02: &lt;10 ⇒ báo thiếu mẫu, không đổi</t>
   </si>
   <si>
-    <t>Theo dõi hiệu năng và báo cáo chất lượng dịch vụ</t>
+    <t>Sổ hiệu năng + báo cáo SLA + quyết toán partner 🔧R1</t>
   </si>
   <si>
     <t>ops/báo-cáo-sla</t>
@@ -809,7 +917,7 @@
     <t>AC01: đúng hạn = đúng giao/nhận đúng hạn; AC02: CSV mở được không cần app</t>
   </si>
   <si>
-    <t>Tích hợp cổng thanh toán SEPay (QR, xác minh 2 bước)</t>
+    <t>SEPay QR + xác thực 2 lớp</t>
   </si>
   <si>
     <t>khách/thanh-toán</t>
@@ -824,7 +932,22 @@
     <t>AC01: thẻ test đủ tiền ⇒ đơn vào engine; AC02: chỉ webhook không confirm ⇒ đơn đứng PENDING; AC03: DB không trường nào chứa thẻ; AC04: cầu T2 bị xóa — XIN APP KEY TỪ TUẦN 5</t>
   </si>
   <si>
-    <t>Hoàn tiền và đối soát giao dịch hằng ngày</t>
+    <t>🆕R1 Cọc + tất toán theo tiến độ</t>
+  </si>
+  <si>
+    <t>khách/thanh-toán · hub/pack (gate)</t>
+  </si>
+  <si>
+    <t>Cọc (cfg %, default 50) xác minh ⇒ vào sản xuất; tất toán tự gửi trước pack; thiếu ⇒ pack gate chặn</t>
+  </si>
+  <si>
+    <t>FR-CUST-012 · BR-PAY-007/008 · SEC-009</t>
+  </si>
+  <si>
+    <t>AC01: chưa cọc ⇒ 0 job; AC02: thiếu tất toán ⇒ pack 409; AC03: ⚠B19/B20 (% + chính sách mất cọc)</t>
+  </si>
+  <si>
+    <t>Hoàn tiền + đối soát</t>
   </si>
   <si>
     <t>ops/hoàn-tiền</t>
@@ -839,7 +962,7 @@
     <t>AC01: 2 lần bấm hoàn ⇒ 1 giao dịch; AC02: file đối soát có tiêu chí lệch; AC03: hoàn xong đơn DELIVERED thành REFUNDED</t>
   </si>
   <si>
-    <t>Deploy ra máy chủ công khai phục vụ demo</t>
+    <t>Máy chủ demo công khai</t>
   </si>
   <si>
     <t>Nhóm Nền tảng</t>
@@ -854,7 +977,7 @@
     <t>AC01: mở URL từ 4G điện thoại chạy; AC02: restore DB trống bằng bản sao lưu trong 15 phút</t>
   </si>
   <si>
-    <t>Chạy in thực tế tại phòng lab đối tác</t>
+    <t>In thật tại lab đối tác</t>
   </si>
   <si>
     <t>Nhóm Xưởng</t>
@@ -872,7 +995,7 @@
     <t>AC01: bảng số thật đủ cột; AC02: MAPE lần đầu tính được</t>
   </si>
   <si>
-    <t>Dọn lỗi, tổng duyệt 3 kịch bản demo, chốt hồ sơ</t>
+    <t>Bug bash + 3 màn kịch bản + hồ sơ chốt</t>
   </si>
   <si>
     <t>mọi màn</t>
@@ -887,7 +1010,7 @@
     <t>AC01: bảng tiến độ sheet này hết dòng "Phải làm" chưa xong; AC02: người không code bấm thử không vướng</t>
   </si>
   <si>
-    <t>Báo cáo đánh giá kết quả thuật toán</t>
+    <t>Báo cáo kết quả thuật toán</t>
   </si>
   <si>
     <t>Bảng + biểu đồ từ RUN-06; số trace về lần chạy + hạt giống; giới hạn</t>
@@ -914,10 +1037,10 @@
     <t>AC01: chỉ làm khi cả 4 cổng tuần 1–6 đậu đúng hạn</t>
   </si>
   <si>
-    <t>54 dòng công việc</t>
-  </si>
-  <si>
-    <t>Lượng việc nằm trong chữ "Cụ thể"; quy đổi ngày công (ẩn): tổng ≈ 172d vs trần 4 người × 8 tuần ≈ 128–160d ⇒ cắt đúng nhóm BỎ-01/Nên-làm khi bất kỳ cổng tuần nào trễ</t>
+    <t>62 dòng công việc</t>
+  </si>
+  <si>
+    <t>Lượng việc nằm trong chữ "Cụ thể"; quy đổi ngày công (ẩn): tổng ≈ 189d vs trần 4 người × 8 tuần ≈ 128–160d ⇒ cắt đúng nhóm BỎ-01/Nên-làm khi bất kỳ cổng tuần nào trễ</t>
   </si>
   <si>
     <t>TÓM TẮT MÀN HÌNH FE — một màn một chủ trong một tuần</t>
@@ -1101,17 +1224,24 @@
       <i/>
       <color rgb="FF7F7F7F"/>
       <sz val="9"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <i/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1564,13 +1694,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K70"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:K78"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
     <col min="3" max="3" width="5" customWidth="1"/>
-    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="4" max="4" width="39.7265625" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="24" customWidth="1"/>
     <col min="7" max="7" width="64" customWidth="1"/>
@@ -1630,7 +1760,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -1665,7 +1795,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -1700,7 +1830,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -1735,7 +1865,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -1770,7 +1900,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -1805,7 +1935,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -1840,7 +1970,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -1875,7 +2005,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -1904,13 +2034,13 @@
         <v>18</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -1921,31 +2051,31 @@
         <v>26</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>28</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I11" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -1956,31 +2086,31 @@
         <v>26</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>28</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -1988,34 +2118,34 @@
         <v>2</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>46</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>18</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -2023,22 +2153,22 @@
         <v>2</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>18</v>
@@ -2047,10 +2177,10 @@
         <v>19</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="15" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -2058,22 +2188,22 @@
         <v>2</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>18</v>
@@ -2082,10 +2212,10 @@
         <v>19</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" ht="43.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -2093,34 +2223,34 @@
         <v>2</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>91</v>
+        <v>38</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>92</v>
       </c>
       <c r="E16" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="G16" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="H16" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="H16" s="6" t="s">
+      <c r="I16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="K16" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I16" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -2128,7 +2258,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>98</v>
@@ -2155,7 +2285,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" ht="43.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -2163,13 +2293,13 @@
         <v>2</v>
       </c>
       <c r="C18" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>46</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>106</v>
@@ -2190,7 +2320,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -2198,22 +2328,22 @@
         <v>2</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>51</v>
+        <v>110</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>46</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>18</v>
@@ -2222,10 +2352,10 @@
         <v>19</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
         <v>18</v>
       </c>
@@ -2236,19 +2366,19 @@
         <v>51</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E20" s="5" t="s">
         <v>46</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I20" s="5" t="s">
         <v>18</v>
@@ -2257,10 +2387,10 @@
         <v>19</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
         <v>19</v>
       </c>
@@ -2268,69 +2398,69 @@
         <v>2</v>
       </c>
       <c r="C21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="K21" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="22" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="5">
+        <v>20</v>
+      </c>
+      <c r="B22" s="5">
+        <v>2</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="E21" s="5" t="s">
+      <c r="D22" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F21" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="I21" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="J21" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="K21" s="6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="7">
-        <v>20</v>
-      </c>
-      <c r="B22" s="7">
-        <v>3</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>126</v>
-      </c>
-      <c r="G22" s="8" t="s">
+      <c r="F22" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H22" s="8" t="s">
+      <c r="G22" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K22" s="8" t="s">
+      <c r="H22" s="6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I22" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="K22" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="23" ht="43.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="7">
         <v>21</v>
       </c>
@@ -2341,19 +2471,19 @@
         <v>26</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E23" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>18</v>
@@ -2362,10 +2492,10 @@
         <v>19</v>
       </c>
       <c r="K23" s="8" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="7">
         <v>22</v>
       </c>
@@ -2376,19 +2506,19 @@
         <v>26</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E24" s="7" t="s">
         <v>28</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>18</v>
@@ -2397,10 +2527,10 @@
         <v>19</v>
       </c>
       <c r="K24" s="8" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="25" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="7">
         <v>23</v>
       </c>
@@ -2408,22 +2538,22 @@
         <v>3</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>26</v>
+        <v>97</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>28</v>
+        <v>142</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>18</v>
@@ -2432,10 +2562,10 @@
         <v>19</v>
       </c>
       <c r="K25" s="8" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="26" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="7">
         <v>24</v>
       </c>
@@ -2443,22 +2573,22 @@
         <v>3</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>86</v>
+        <v>142</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>18</v>
@@ -2467,10 +2597,10 @@
         <v>19</v>
       </c>
       <c r="K26" s="8" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="27" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
         <v>25</v>
       </c>
@@ -2478,22 +2608,22 @@
         <v>3</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>84</v>
+        <v>26</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>150</v>
+        <v>28</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>18</v>
@@ -2502,10 +2632,10 @@
         <v>19</v>
       </c>
       <c r="K27" s="8" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="28" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="7">
         <v>26</v>
       </c>
@@ -2513,22 +2643,22 @@
         <v>3</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>91</v>
+        <v>26</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>18</v>
@@ -2537,10 +2667,10 @@
         <v>19</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="29" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="7">
         <v>27</v>
       </c>
@@ -2548,22 +2678,22 @@
         <v>3</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>91</v>
+        <v>26</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>18</v>
@@ -2572,10 +2702,10 @@
         <v>19</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="7">
         <v>28</v>
       </c>
@@ -2583,22 +2713,22 @@
         <v>3</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>46</v>
+        <v>87</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I30" s="7" t="s">
         <v>18</v>
@@ -2607,10 +2737,10 @@
         <v>19</v>
       </c>
       <c r="K30" s="8" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="7">
         <v>29</v>
       </c>
@@ -2618,22 +2748,22 @@
         <v>3</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>46</v>
+        <v>171</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="I31" s="7" t="s">
         <v>18</v>
@@ -2642,10 +2772,10 @@
         <v>19</v>
       </c>
       <c r="K31" s="8" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="32" ht="43.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" s="7">
         <v>30</v>
       </c>
@@ -2653,174 +2783,174 @@
         <v>3</v>
       </c>
       <c r="C32" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>176</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="H32" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J32" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="33" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="7">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7">
+        <v>3</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="H33" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="34" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="7">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7">
+        <v>3</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="7">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7">
+        <v>3</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="36" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="7">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7">
+        <v>3</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D32" s="7" t="s">
-        <v>174</v>
-      </c>
-      <c r="E32" s="7" t="s">
+      <c r="D36" s="7" t="s">
+        <v>195</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F32" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="G32" s="8" t="s">
-        <v>176</v>
-      </c>
-      <c r="H32" s="8" t="s">
-        <v>177</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="J32" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="K32" s="8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="9">
-        <v>31</v>
-      </c>
-      <c r="B33" s="9">
-        <v>4</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>182</v>
-      </c>
-      <c r="I33" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J33" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K33" s="10" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="9">
-        <v>32</v>
-      </c>
-      <c r="B34" s="9">
-        <v>4</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" s="9" t="s">
-        <v>184</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F34" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="H34" s="10" t="s">
-        <v>187</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J34" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K34" s="10" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="9">
-        <v>33</v>
-      </c>
-      <c r="B35" s="9">
-        <v>4</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F35" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="G35" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>193</v>
-      </c>
-      <c r="I35" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J35" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K35" s="10" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="9">
-        <v>34</v>
-      </c>
-      <c r="B36" s="9">
-        <v>4</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="F36" s="10" t="s">
+      <c r="F36" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="G36" s="10" t="s">
+      <c r="G36" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="H36" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="I36" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J36" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K36" s="10" t="s">
+      <c r="I36" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K36" s="8" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="9">
         <v>35</v>
       </c>
@@ -2828,7 +2958,7 @@
         <v>4</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>189</v>
+        <v>38</v>
       </c>
       <c r="D37" s="9" t="s">
         <v>200</v>
@@ -2855,7 +2985,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="9">
         <v>36</v>
       </c>
@@ -2863,13 +2993,13 @@
         <v>4</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>84</v>
+        <v>38</v>
       </c>
       <c r="D38" s="9" t="s">
         <v>205</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="F38" s="10" t="s">
         <v>206</v>
@@ -2890,7 +3020,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="9">
         <v>37</v>
       </c>
@@ -2898,22 +3028,22 @@
         <v>4</v>
       </c>
       <c r="C39" s="9" t="s">
-        <v>84</v>
+        <v>210</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I39" s="9" t="s">
         <v>18</v>
@@ -2922,10 +3052,10 @@
         <v>19</v>
       </c>
       <c r="K39" s="10" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="40" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
         <v>38</v>
       </c>
@@ -2933,22 +3063,22 @@
         <v>4</v>
       </c>
       <c r="C40" s="9" t="s">
-        <v>84</v>
+        <v>210</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E40" s="9" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H40" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I40" s="9" t="s">
         <v>18</v>
@@ -2957,10 +3087,10 @@
         <v>19</v>
       </c>
       <c r="K40" s="10" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="41" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="9">
         <v>39</v>
       </c>
@@ -2968,13 +3098,13 @@
         <v>4</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>221</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>79</v>
+        <v>40</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>222</v>
@@ -2995,7 +3125,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="9">
         <v>40</v>
       </c>
@@ -3003,22 +3133,22 @@
         <v>4</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>26</v>
+        <v>85</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>226</v>
       </c>
       <c r="E42" s="9" t="s">
-        <v>28</v>
+        <v>87</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>131</v>
+        <v>227</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H42" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I42" s="9" t="s">
         <v>18</v>
@@ -3027,7 +3157,7 @@
         <v>19</v>
       </c>
       <c r="K42" s="10" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -3038,710 +3168,988 @@
         <v>4</v>
       </c>
       <c r="C43" s="9" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E43" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="G43" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="H43" s="10" t="s">
+        <v>234</v>
+      </c>
+      <c r="I43" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J43" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K43" s="10" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="44" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="9">
+        <v>42</v>
+      </c>
+      <c r="B44" s="9">
+        <v>4</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>237</v>
+      </c>
+      <c r="G44" s="10" t="s">
+        <v>238</v>
+      </c>
+      <c r="H44" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="I44" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J44" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K44" s="10" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="45" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="9">
+        <v>43</v>
+      </c>
+      <c r="B45" s="9">
+        <v>4</v>
+      </c>
+      <c r="C45" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="G45" s="10" t="s">
+        <v>242</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>243</v>
+      </c>
+      <c r="I45" s="9"/>
+      <c r="J45" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K45" s="10" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="46" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="9">
+        <v>44</v>
+      </c>
+      <c r="B46" s="9">
+        <v>4</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>246</v>
+      </c>
+      <c r="G46" s="10" t="s">
+        <v>247</v>
+      </c>
+      <c r="H46" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="I46" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J46" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K46" s="10" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="47" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="9">
+        <v>45</v>
+      </c>
+      <c r="B47" s="9">
+        <v>4</v>
+      </c>
+      <c r="C47" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F47" s="10" t="s">
+        <v>252</v>
+      </c>
+      <c r="G47" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="H47" s="10" t="s">
+        <v>254</v>
+      </c>
+      <c r="I47" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J47" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K47" s="10" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="48" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="9">
         <v>46</v>
       </c>
-      <c r="F43" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="G43" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="I43" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J43" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K43" s="10" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="11">
-        <v>42</v>
-      </c>
-      <c r="B44" s="11">
+      <c r="B48" s="9">
+        <v>4</v>
+      </c>
+      <c r="C48" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F48" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="G48" s="10" t="s">
+        <v>257</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>258</v>
+      </c>
+      <c r="I48" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J48" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K48" s="10" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="49" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" s="9">
+        <v>47</v>
+      </c>
+      <c r="B49" s="9">
+        <v>4</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F49" s="10" t="s">
+        <v>261</v>
+      </c>
+      <c r="G49" s="10" t="s">
+        <v>262</v>
+      </c>
+      <c r="H49" s="10" t="s">
+        <v>263</v>
+      </c>
+      <c r="I49" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="J49" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="K49" s="10" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="50" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="11">
+        <v>48</v>
+      </c>
+      <c r="B50" s="11">
         <v>5</v>
       </c>
-      <c r="C44" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="D44" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="E44" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="F44" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="G44" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="H44" s="12" t="s">
-        <v>240</v>
-      </c>
-      <c r="I44" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J44" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="K44" s="12" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="11">
-        <v>43</v>
-      </c>
-      <c r="B45" s="11">
+      <c r="C50" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="F50" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="G50" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="I50" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J50" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K50" s="12" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="51" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="11">
+        <v>49</v>
+      </c>
+      <c r="B51" s="11">
         <v>5</v>
       </c>
-      <c r="C45" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="F45" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="G45" s="12" t="s">
-        <v>243</v>
-      </c>
-      <c r="H45" s="12" t="s">
-        <v>244</v>
-      </c>
-      <c r="I45" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J45" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="K45" s="12" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="11">
-        <v>44</v>
-      </c>
-      <c r="B46" s="11">
+      <c r="C51" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>272</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="F51" s="12" t="s">
+        <v>268</v>
+      </c>
+      <c r="G51" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="I51" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J51" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K51" s="12" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="52" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="11">
+        <v>50</v>
+      </c>
+      <c r="B52" s="11">
         <v>5</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C52" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="D46" s="11" t="s">
-        <v>246</v>
-      </c>
-      <c r="E46" s="11" t="s">
+      <c r="D52" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="E52" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="F46" s="12" t="s">
-        <v>247</v>
-      </c>
-      <c r="G46" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="H46" s="12" t="s">
-        <v>249</v>
-      </c>
-      <c r="I46" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J46" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="K46" s="12" t="s">
+      <c r="F52" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="G52" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="H52" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="I52" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="K52" s="12" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="53" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="13">
+        <v>51</v>
+      </c>
+      <c r="B53" s="13">
+        <v>6</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="F53" s="14" t="s">
+        <v>268</v>
+      </c>
+      <c r="G53" s="14" t="s">
+        <v>282</v>
+      </c>
+      <c r="H53" s="14" t="s">
+        <v>283</v>
+      </c>
+      <c r="I53" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J53" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K53" s="14" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="54" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="13">
+        <v>52</v>
+      </c>
+      <c r="B54" s="13">
+        <v>6</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="H54" s="14" t="s">
+        <v>288</v>
+      </c>
+      <c r="I54" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J54" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K54" s="14" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="55" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="13">
+        <v>53</v>
+      </c>
+      <c r="B55" s="13">
+        <v>6</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>290</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F55" s="14" t="s">
+        <v>291</v>
+      </c>
+      <c r="G55" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="H55" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="I55" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J55" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K55" s="14" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="56" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="13">
+        <v>54</v>
+      </c>
+      <c r="B56" s="13">
+        <v>6</v>
+      </c>
+      <c r="C56" s="13" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="13">
-        <v>45</v>
-      </c>
-      <c r="B47" s="13">
-        <v>6</v>
-      </c>
-      <c r="C47" s="13" t="s">
-        <v>235</v>
-      </c>
-      <c r="D47" s="13" t="s">
-        <v>251</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>237</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>238</v>
-      </c>
-      <c r="G47" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="H47" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="I47" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J47" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K47" s="14" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="13">
+      <c r="D56" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="F56" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="G56" s="14" t="s">
+        <v>297</v>
+      </c>
+      <c r="H56" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="I56" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="J56" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="K56" s="14" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="57" ht="43.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="15">
+        <v>55</v>
+      </c>
+      <c r="B57" s="15">
+        <v>7</v>
+      </c>
+      <c r="C57" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D57" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="E57" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="B48" s="13">
-        <v>6</v>
-      </c>
-      <c r="C48" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="D48" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="E48" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="F48" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="G48" s="14" t="s">
-        <v>257</v>
-      </c>
-      <c r="H48" s="14" t="s">
-        <v>258</v>
-      </c>
-      <c r="I48" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J48" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K48" s="14" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="13">
-        <v>47</v>
-      </c>
-      <c r="B49" s="13">
-        <v>6</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D49" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="F49" s="14" t="s">
-        <v>261</v>
-      </c>
-      <c r="G49" s="14" t="s">
-        <v>262</v>
-      </c>
-      <c r="H49" s="14" t="s">
-        <v>263</v>
-      </c>
-      <c r="I49" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="J49" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="K49" s="14" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="15">
-        <v>48</v>
-      </c>
-      <c r="B50" s="15">
+      <c r="F57" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="G57" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="H57" s="16" t="s">
+        <v>303</v>
+      </c>
+      <c r="I57" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J57" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K57" s="16" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="58" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="15">
+        <v>56</v>
+      </c>
+      <c r="B58" s="15">
         <v>7</v>
       </c>
-      <c r="C50" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D50" s="15" t="s">
+      <c r="C58" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="E58" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="F58" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="G58" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="H58" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="I58" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J58" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K58" s="16" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="59" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="15">
+        <v>57</v>
+      </c>
+      <c r="B59" s="15">
+        <v>7</v>
+      </c>
+      <c r="C59" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D59" s="15" t="s">
+        <v>310</v>
+      </c>
+      <c r="E59" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="F59" s="16" t="s">
+        <v>311</v>
+      </c>
+      <c r="G59" s="16" t="s">
+        <v>312</v>
+      </c>
+      <c r="H59" s="16" t="s">
+        <v>313</v>
+      </c>
+      <c r="I59" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J59" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K59" s="16" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="60" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" s="15">
+        <v>58</v>
+      </c>
+      <c r="B60" s="15">
+        <v>7</v>
+      </c>
+      <c r="C60" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" s="15" t="s">
+        <v>315</v>
+      </c>
+      <c r="E60" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="F60" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="G60" s="16" t="s">
+        <v>317</v>
+      </c>
+      <c r="H60" s="16" t="s">
+        <v>318</v>
+      </c>
+      <c r="I60" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J60" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K60" s="16" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="61" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="15">
+        <v>59</v>
+      </c>
+      <c r="B61" s="15">
+        <v>7</v>
+      </c>
+      <c r="C61" s="15" t="s">
         <v>265</v>
       </c>
-      <c r="E50" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F50" s="16" t="s">
-        <v>266</v>
-      </c>
-      <c r="G50" s="16" t="s">
+      <c r="D61" s="15" t="s">
+        <v>320</v>
+      </c>
+      <c r="E61" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="F61" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="G61" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="H61" s="16" t="s">
+        <v>324</v>
+      </c>
+      <c r="I61" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="J61" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="K61" s="16" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="62" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="17">
+        <v>60</v>
+      </c>
+      <c r="B62" s="17">
+        <v>8</v>
+      </c>
+      <c r="C62" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="D62" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="E62" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="G62" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="H62" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="I62" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J62" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K62" s="18" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="63" ht="29" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="17">
+        <v>61</v>
+      </c>
+      <c r="B63" s="17">
+        <v>8</v>
+      </c>
+      <c r="C63" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="D63" s="17" t="s">
+        <v>331</v>
+      </c>
+      <c r="E63" s="17" t="s">
         <v>267</v>
       </c>
-      <c r="H50" s="16" t="s">
-        <v>268</v>
-      </c>
-      <c r="I50" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J50" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K50" s="16" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="15">
-        <v>49</v>
-      </c>
-      <c r="B51" s="15">
-        <v>7</v>
-      </c>
-      <c r="C51" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D51" s="15" t="s">
-        <v>270</v>
-      </c>
-      <c r="E51" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="F51" s="16" t="s">
-        <v>271</v>
-      </c>
-      <c r="G51" s="16" t="s">
-        <v>272</v>
-      </c>
-      <c r="H51" s="16" t="s">
-        <v>273</v>
-      </c>
-      <c r="I51" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J51" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K51" s="16" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" s="15">
-        <v>50</v>
-      </c>
-      <c r="B52" s="15">
-        <v>7</v>
-      </c>
-      <c r="C52" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="D52" s="15" t="s">
-        <v>275</v>
-      </c>
-      <c r="E52" s="15" t="s">
-        <v>276</v>
-      </c>
-      <c r="F52" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="G52" s="16" t="s">
-        <v>277</v>
-      </c>
-      <c r="H52" s="16" t="s">
-        <v>278</v>
-      </c>
-      <c r="I52" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J52" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K52" s="16" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="15">
+      <c r="F63" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="G63" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="H63" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="I63" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="J63" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="K63" s="18" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="64" ht="43.5" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>62</v>
+      </c>
+      <c r="B64" t="s">
+        <v>127</v>
+      </c>
+      <c r="C64" t="s">
         <v>51</v>
       </c>
-      <c r="B53" s="15">
-        <v>7</v>
-      </c>
-      <c r="C53" s="15" t="s">
-        <v>235</v>
-      </c>
-      <c r="D53" s="15" t="s">
-        <v>280</v>
-      </c>
-      <c r="E53" s="15" t="s">
-        <v>281</v>
-      </c>
-      <c r="F53" s="16" t="s">
-        <v>282</v>
-      </c>
-      <c r="G53" s="16" t="s">
-        <v>283</v>
-      </c>
-      <c r="H53" s="16" t="s">
-        <v>284</v>
-      </c>
-      <c r="I53" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="J53" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="K53" s="16" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A54" s="17">
-        <v>52</v>
-      </c>
-      <c r="B54" s="17">
-        <v>8</v>
-      </c>
-      <c r="C54" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="D54" s="17" t="s">
-        <v>286</v>
-      </c>
-      <c r="E54" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="F54" s="18" t="s">
-        <v>287</v>
-      </c>
-      <c r="G54" s="18" t="s">
-        <v>288</v>
-      </c>
-      <c r="H54" s="18" t="s">
-        <v>289</v>
-      </c>
-      <c r="I54" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J54" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="K54" s="18" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" s="17">
-        <v>53</v>
-      </c>
-      <c r="B55" s="17">
-        <v>8</v>
-      </c>
-      <c r="C55" s="17" t="s">
-        <v>235</v>
-      </c>
-      <c r="D55" s="17" t="s">
-        <v>291</v>
-      </c>
-      <c r="E55" s="17" t="s">
-        <v>237</v>
-      </c>
-      <c r="F55" s="18" t="s">
-        <v>121</v>
-      </c>
-      <c r="G55" s="18" t="s">
-        <v>292</v>
-      </c>
-      <c r="H55" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="I55" s="17" t="s">
-        <v>18</v>
-      </c>
-      <c r="J55" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="K55" s="18" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56">
-        <v>54</v>
-      </c>
-      <c r="B56" t="s">
-        <v>121</v>
-      </c>
-      <c r="C56" t="s">
-        <v>51</v>
-      </c>
-      <c r="D56" t="s">
-        <v>295</v>
-      </c>
-      <c r="E56" t="s">
-        <v>121</v>
-      </c>
-      <c r="F56" s="19" t="s">
-        <v>296</v>
-      </c>
-      <c r="G56" s="19" t="s">
-        <v>297</v>
-      </c>
-      <c r="H56" s="19" t="s">
-        <v>298</v>
-      </c>
-      <c r="I56" t="s">
-        <v>18</v>
-      </c>
-      <c r="J56" t="s">
-        <v>19</v>
-      </c>
-      <c r="K56" s="19" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D57" s="20" t="s">
-        <v>300</v>
-      </c>
-      <c r="E57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="F57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="G57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="H57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="I57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="J57" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="K57" s="20" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="C59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="D59" s="20" t="s">
-        <v>302</v>
-      </c>
-      <c r="E59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="F59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="G59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="H59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="I59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="J59" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="K59" s="20" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="60" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D60" s="21" t="s">
-        <v>303</v>
-      </c>
-      <c r="E60" s="21" t="s">
-        <v>304</v>
-      </c>
-      <c r="F60" s="21" t="s">
-        <v>305</v>
-      </c>
-      <c r="G60" s="21" t="s">
+      <c r="D64" t="s">
+        <v>335</v>
+      </c>
+      <c r="E64" t="s">
+        <v>127</v>
+      </c>
+      <c r="F64" s="19" t="s">
+        <v>336</v>
+      </c>
+      <c r="G64" s="19" t="s">
+        <v>337</v>
+      </c>
+      <c r="H64" s="19" t="s">
+        <v>338</v>
+      </c>
+      <c r="I64" t="s">
+        <v>18</v>
+      </c>
+      <c r="J64" t="s">
+        <v>19</v>
+      </c>
+      <c r="K64" s="19" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65" s="20" t="s">
+        <v>340</v>
+      </c>
+      <c r="E65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="G65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="I65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="J65" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="K65" s="20" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="D67" s="20" t="s">
+        <v>342</v>
+      </c>
+      <c r="E67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="G67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="H67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="I67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="J67" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="K67" s="20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D68" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="E68" s="21" t="s">
+        <v>344</v>
+      </c>
+      <c r="F68" s="21" t="s">
+        <v>345</v>
+      </c>
+      <c r="G68" s="21" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D61" s="22" t="s">
-        <v>306</v>
-      </c>
-      <c r="E61" t="s">
-        <v>307</v>
-      </c>
-      <c r="F61" s="22" t="s">
-        <v>308</v>
-      </c>
-      <c r="G61" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="62" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D62" s="22" t="s">
-        <v>310</v>
-      </c>
-      <c r="E62" t="s">
-        <v>307</v>
-      </c>
-      <c r="F62" s="22" t="s">
-        <v>311</v>
-      </c>
-      <c r="G62" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="63" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D63" s="22" t="s">
-        <v>313</v>
-      </c>
-      <c r="E63" t="s">
-        <v>314</v>
-      </c>
-      <c r="F63" s="22" t="s">
-        <v>315</v>
-      </c>
-      <c r="G63" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="64" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D64" s="22" t="s">
-        <v>317</v>
-      </c>
-      <c r="E64" t="s">
-        <v>318</v>
-      </c>
-      <c r="F64" s="22" t="s">
-        <v>319</v>
-      </c>
-      <c r="G64" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="65" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D65" s="22" t="s">
-        <v>321</v>
-      </c>
-      <c r="E65" t="s">
-        <v>318</v>
-      </c>
-      <c r="F65" s="22" t="s">
-        <v>322</v>
-      </c>
-      <c r="G65" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="66" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D66" s="22" t="s">
-        <v>324</v>
-      </c>
-      <c r="E66" t="s">
-        <v>325</v>
-      </c>
-      <c r="F66" s="22" t="s">
-        <v>326</v>
-      </c>
-      <c r="G66" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="67" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D67" s="22" t="s">
-        <v>328</v>
-      </c>
-      <c r="E67" t="s">
-        <v>329</v>
-      </c>
-      <c r="F67" s="22" t="s">
-        <v>330</v>
-      </c>
-      <c r="G67" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="68" spans="4:7" x14ac:dyDescent="0.25">
-      <c r="D68" s="22" t="s">
-        <v>332</v>
-      </c>
-      <c r="E68" t="s">
-        <v>333</v>
-      </c>
-      <c r="F68" s="22" t="s">
-        <v>334</v>
-      </c>
-      <c r="G68" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="69" spans="4:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D69" s="22" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="E69" t="s">
-        <v>336</v>
+        <v>347</v>
       </c>
       <c r="F69" s="22" t="s">
-        <v>337</v>
+        <v>348</v>
       </c>
       <c r="G69" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="70" spans="4:7" x14ac:dyDescent="0.25">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="D70" s="22" t="s">
-        <v>339</v>
+        <v>350</v>
       </c>
       <c r="E70" t="s">
-        <v>307</v>
+        <v>347</v>
       </c>
       <c r="F70" s="22" t="s">
-        <v>340</v>
+        <v>351</v>
       </c>
       <c r="G70" t="s">
-        <v>309</v>
+        <v>352</v>
+      </c>
+    </row>
+    <row r="71" ht="29" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D71" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="E71" t="s">
+        <v>354</v>
+      </c>
+      <c r="F71" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="G71" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="72" ht="29" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D72" s="22" t="s">
+        <v>357</v>
+      </c>
+      <c r="E72" t="s">
+        <v>358</v>
+      </c>
+      <c r="F72" s="22" t="s">
+        <v>359</v>
+      </c>
+      <c r="G72" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D73" s="22" t="s">
+        <v>361</v>
+      </c>
+      <c r="E73" t="s">
+        <v>358</v>
+      </c>
+      <c r="F73" s="22" t="s">
+        <v>362</v>
+      </c>
+      <c r="G73" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D74" s="22" t="s">
+        <v>364</v>
+      </c>
+      <c r="E74" t="s">
+        <v>365</v>
+      </c>
+      <c r="F74" s="22" t="s">
+        <v>366</v>
+      </c>
+      <c r="G74" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="75" ht="29" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D75" s="22" t="s">
+        <v>368</v>
+      </c>
+      <c r="E75" t="s">
+        <v>369</v>
+      </c>
+      <c r="F75" s="22" t="s">
+        <v>370</v>
+      </c>
+      <c r="G75" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="76" ht="29" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D76" s="22" t="s">
+        <v>372</v>
+      </c>
+      <c r="E76" t="s">
+        <v>373</v>
+      </c>
+      <c r="F76" s="22" t="s">
+        <v>374</v>
+      </c>
+      <c r="G76" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="77" ht="29" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D77" s="22" t="s">
+        <v>375</v>
+      </c>
+      <c r="E77" t="s">
+        <v>376</v>
+      </c>
+      <c r="F77" s="22" t="s">
+        <v>377</v>
+      </c>
+      <c r="G77" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="78" ht="29" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D78" s="22" t="s">
+        <v>379</v>
+      </c>
+      <c r="E78" t="s">
+        <v>347</v>
+      </c>
+      <c r="F78" s="22" t="s">
+        <v>380</v>
+      </c>
+      <c r="G78" t="s">
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -3750,28 +4158,28 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" sqref="I10:I56">
+    <dataValidation type="list" allowBlank="1" sqref="I10:I64">
       <formula1>"Tân,Minh,Nhật,Tuấn"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="I3:I56">
+    <dataValidation type="list" allowBlank="1" sqref="I3:I64">
       <formula1>"Tân,Minh,Nhật,Tuấn"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J10:J56">
+    <dataValidation type="list" allowBlank="1" sqref="J10:J64">
       <formula1>"Chưa làm,Đang làm,Xong,Bỏ qua"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="J3:J56">
+    <dataValidation type="list" allowBlank="1" sqref="J3:J64">
       <formula1>"Chưa làm,Đang làm,Xong,Bỏ qua"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3780,174 +4188,210 @@
   <sheetData>
     <row r="1" spans="1:10" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>341</v>
+        <v>381</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>342</v>
+        <v>382</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>343</v>
+        <v>383</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>344</v>
+        <v>384</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>345</v>
+        <v>385</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>346</v>
+        <v>386</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>347</v>
+        <v>387</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>348</v>
+        <v>388</v>
       </c>
       <c r="I1" s="20" t="s">
-        <v>349</v>
+        <v>389</v>
       </c>
       <c r="J1" s="20" t="s">
-        <v>350</v>
+        <v>390</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>351</v>
+        <v>391</v>
       </c>
       <c r="B2">
         <f>SUM(C2:J2)</f>
+        <v>0</v>
       </c>
       <c r="C2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,1)</f>
+        <v>0</v>
       </c>
       <c r="D2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,2)</f>
+        <v>0</v>
       </c>
       <c r="E2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,3)</f>
+        <v>0</v>
       </c>
       <c r="F2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,4)</f>
+        <v>0</v>
       </c>
       <c r="G2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,5)</f>
+        <v>0</v>
       </c>
       <c r="H2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,6)</f>
+        <v>0</v>
       </c>
       <c r="I2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,7)</f>
+        <v>0</v>
       </c>
       <c r="J2">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A2,'PHÂN CÔNG — 1 TRANG'!$B:$B,8)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>352</v>
+        <v>392</v>
       </c>
       <c r="B3">
         <f>SUM(C3:J3)</f>
+        <v>0</v>
       </c>
       <c r="C3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,1)</f>
+        <v>0</v>
       </c>
       <c r="D3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,2)</f>
+        <v>0</v>
       </c>
       <c r="E3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,3)</f>
+        <v>0</v>
       </c>
       <c r="F3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,4)</f>
+        <v>0</v>
       </c>
       <c r="G3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,5)</f>
+        <v>0</v>
       </c>
       <c r="H3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,6)</f>
+        <v>0</v>
       </c>
       <c r="I3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,7)</f>
+        <v>0</v>
       </c>
       <c r="J3">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A3,'PHÂN CÔNG — 1 TRANG'!$B:$B,8)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>353</v>
+        <v>393</v>
       </c>
       <c r="B4">
         <f>SUM(C4:J4)</f>
+        <v>0</v>
       </c>
       <c r="C4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,1)</f>
+        <v>0</v>
       </c>
       <c r="D4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,2)</f>
+        <v>0</v>
       </c>
       <c r="E4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,3)</f>
+        <v>0</v>
       </c>
       <c r="F4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,4)</f>
+        <v>0</v>
       </c>
       <c r="G4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,5)</f>
+        <v>0</v>
       </c>
       <c r="H4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,6)</f>
+        <v>0</v>
       </c>
       <c r="I4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,7)</f>
+        <v>0</v>
       </c>
       <c r="J4">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A4,'PHÂN CÔNG — 1 TRANG'!$B:$B,8)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>354</v>
+        <v>394</v>
       </c>
       <c r="B5">
         <f>SUM(C5:J5)</f>
+        <v>0</v>
       </c>
       <c r="C5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,1)</f>
+        <v>0</v>
       </c>
       <c r="D5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,2)</f>
+        <v>0</v>
       </c>
       <c r="E5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,3)</f>
+        <v>0</v>
       </c>
       <c r="F5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,4)</f>
+        <v>0</v>
       </c>
       <c r="G5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,5)</f>
+        <v>0</v>
       </c>
       <c r="H5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,6)</f>
+        <v>0</v>
       </c>
       <c r="I5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,7)</f>
+        <v>0</v>
       </c>
       <c r="J5">
         <f>COUNTIFS('PHÂN CÔNG — 1 TRANG'!$I:$I,$A5,'PHÂN CÔNG — 1 TRANG'!$B:$B,8)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>355</v>
+        <v>395</v>
       </c>
       <c r="B7" t="s">
-        <v>356</v>
+        <v>396</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>